<commit_message>
update regression tests again
</commit_message>
<xml_diff>
--- a/tests/traces/h100/google_owlv2-large-patch14-ensemble__1016001_perf_report.xlsx
+++ b/tests/traces/h100/google_owlv2-large-patch14-ensemble__1016001_perf_report.xlsx
@@ -2069,7 +2069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ6"/>
+  <dimension ref="A1:AJ5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>768</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2284,34 +2284,34 @@
         <v>7.68e-07</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0029296875</v>
+        <v>0.001466751098632812</v>
       </c>
       <c r="H2" t="n">
-        <v>0.25</v>
+        <v>0.4993498049414825</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0009726418028326389</v>
+        <v>0.0004862886133149629</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0009558318314951775</v>
+        <v>0.0004904358115998443</v>
       </c>
       <c r="K2" t="n">
-        <v>7.280491932446589e-05</v>
+        <v>3.557215699598599e-05</v>
       </c>
       <c r="L2" t="n">
-        <v>0.0008651022344448264</v>
+        <v>0.0004331143348229632</v>
       </c>
       <c r="M2" t="n">
-        <v>0.001078689412773253</v>
+        <v>0.0005400469781397342</v>
       </c>
       <c r="N2" t="n">
-        <v>0.0002431604507081597</v>
+        <v>0.0002428281242040907</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0002389579578737944</v>
+        <v>0.0002448990268586999</v>
       </c>
       <c r="P2" t="n">
-        <v>1.820122983111647e-05</v>
+        <v>1.77629496572934e-05</v>
       </c>
       <c r="Q2" t="n">
         <v>0.0002162755586112066</v>
@@ -2341,12 +2341,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::reduce_kernel&lt;512, 1, at::native::ReduceOp&lt;c10::BFloat16, at::native::NormTwoOps&lt;c10::BFloat16, float, c10::BFloat16&gt;, unsigned int, c10::BFloat16, 4&gt; &gt;(at::native::ReduceOp&lt;c10::BFloat16, at::native::NormTwoOps&lt;c10::BFloat16, float, c10::BFloat16&gt;, unsigned int, c10::BFloat16, 4&gt;)', 'stream': 7, 'count': 10, 'total_duration_us': np.float64(31.743), 'mean_duration_us': np.float64(3.1742999999999997), 'median_duration_us': np.float64(3.216), 'std_dev_duration_us': np.float64(0.22374005005809758), 'min_duration_us': np.float64(2.848), 'max_duration_us': np.float64(3.551)}]</t>
+          <t>[{'name': 'void at::native::reduce_kernel&lt;512, 1, at::native::ReduceOp&lt;c10::BFloat16, at::native::NormTwoOps&lt;c10::BFloat16, float, c10::BFloat16&gt;, unsigned int, c10::BFloat16, 4&gt; &gt;(at::native::ReduceOp&lt;c10::BFloat16, at::native::NormTwoOps&lt;c10::BFloat16, float, c10::BFloat16&gt;, unsigned int, c10::BFloat16, 4&gt;)', 'stream': 7, 'count': 15, 'total_duration_us': np.float64(47.679), 'mean_duration_us': np.float64(3.1786000000000003), 'median_duration_us': np.float64(3.136), 'std_dev_duration_us': np.float64(0.22485248497626176), 'min_duration_us': np.float64(2.848), 'max_duration_us': np.float64(3.551)}]</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::reduce_kernel&lt;512, 1, at::native::ReduceOp&lt;c10:...', 'stream': 7, 'mean_duration_us': np.float64(3.17)}]</t>
+          <t>[{'name': 'void at::native::reduce_kernel&lt;512, 1, at::native::ReduceOp&lt;c10:...', 'stream': 7, 'mean_duration_us': np.float64(3.18)}]</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -2370,13 +2370,13 @@
         </is>
       </c>
       <c r="AC2" t="n">
-        <v>3.174267578125</v>
+        <v>3.178597005208333</v>
       </c>
       <c r="AD2" t="n">
-        <v>3.2159423828125</v>
+        <v>3.135986328125</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.2358569953110188</v>
+        <v>0.2327518180455004</v>
       </c>
       <c r="AF2" t="n">
         <v>2.847900390625</v>
@@ -2385,10 +2385,10 @@
         <v>3.551025390625</v>
       </c>
       <c r="AH2" t="n">
-        <v>31.74267578125</v>
+        <v>47.678955078125</v>
       </c>
       <c r="AI2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="AJ2" t="n">
         <v>4506</v>
@@ -2537,12 +2537,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>aten::linalg_norm</t>
+          <t>aten::max</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>768</t>
+          <t>5184</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2552,53 +2552,33 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>('c10::BFloat16', None)</t>
+          <t>('float', None)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>norm</t>
+          <t>max</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>7.68e-07</v>
+        <v>5.184e-06</v>
       </c>
       <c r="G4" t="n">
-        <v>0.001466751098632812</v>
+        <v>0.01977920532226562</v>
       </c>
       <c r="H4" t="n">
-        <v>0.4993498049414825</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.0004849575764314781</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.0004954890671700488</v>
-      </c>
-      <c r="K4" t="n">
-        <v>3.789683268713756e-05</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.000440935675789179</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.0005224021892362551</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.0002421634711959526</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.000247422369042001</v>
-      </c>
-      <c r="P4" t="n">
-        <v>1.892377601022212e-05</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.0002201811436970673</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0.0002608614312961274</v>
-      </c>
+        <v>0.2499517839922854</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
           <t>python3</t>
@@ -2616,62 +2596,58 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>vector_bf16</t>
+          <t>vector_fp32</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>[{'name': 'void at::native::reduce_kernel&lt;512, 1, at::native::ReduceOp&lt;c10::BFloat16, at::native::NormTwoOps&lt;c10::BFloat16, float, c10::BFloat16&gt;, unsigned int, c10::BFloat16, 4&gt; &gt;(at::native::ReduceOp&lt;c10::BFloat16, at::native::NormTwoOps&lt;c10::BFloat16, float, c10::BFloat16&gt;, unsigned int, c10::BFloat16, 4&gt;)', 'stream': 7, 'count': 5, 'total_duration_us': np.float64(15.936), 'mean_duration_us': np.float64(3.1872), 'median_duration_us': np.float64(3.104), 'std_dev_duration_us': np.float64(0.2268165778773677), 'min_duration_us': np.float64(2.944), 'max_duration_us': np.float64(3.488)}]</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>[{'name': 'void at::native::reduce_kernel&lt;512, 1, at::native::ReduceOp&lt;c10:...', 'stream': 7, 'mean_duration_us': np.float64(3.19)}]</t>
-        </is>
-      </c>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>[[1, 1, 768], [], [], [], []]</t>
+          <t>[[1, 5184, 1], [], []]</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>['c10::BFloat16', '', 'ScalarList', 'Scalar', '']</t>
+          <t>['float', 'Scalar', 'Scalar']</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>[[768, 768, 1], [], [], [], []]</t>
+          <t>[[5184, 1, 1], [], []]</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>['', '', '[-1]', 'True', '']</t>
+          <t>['', '-1', 'False']</t>
         </is>
       </c>
       <c r="AC4" t="n">
-        <v>3.187255859375</v>
+        <v>0</v>
       </c>
       <c r="AD4" t="n">
-        <v>3.10400390625</v>
+        <v>0</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.2535787377464963</v>
+        <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>2.944091796875</v>
+        <v>0</v>
       </c>
       <c r="AG4" t="n">
-        <v>3.488037109375</v>
+        <v>0</v>
       </c>
       <c r="AH4" t="n">
-        <v>15.936279296875</v>
+        <v>0</v>
       </c>
       <c r="AI4" t="n">
         <v>5</v>
       </c>
       <c r="AJ4" t="n">
-        <v>4581</v>
+        <v>23754</v>
       </c>
     </row>
     <row r="5">
@@ -2682,17 +2658,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>5184</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5184</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>('float', None)</t>
+          <t>('int', None)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2701,14 +2677,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>5.184e-06</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.03955078125</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.125</v>
-      </c>
+        <v>1e-09</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -2734,11 +2706,7 @@
           <t>thread 21587 (python3)</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>vector_fp32</t>
-        </is>
-      </c>
+      <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr">
         <is>
           <t>[]</t>
@@ -2747,22 +2715,22 @@
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>[[1, 5184, 1], [], []]</t>
+          <t>[[1], [1]]</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>['float', 'Scalar', 'Scalar']</t>
+          <t>['int', 'int']</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>[[5184, 1, 1], [], []]</t>
+          <t>[[2], [2]]</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>['', '-1', 'False']</t>
+          <t>['', '']</t>
         </is>
       </c>
       <c r="AC5" t="n">
@@ -2787,114 +2755,6 @@
         <v>5</v>
       </c>
       <c r="AJ5" t="n">
-        <v>23754</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>aten::max</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>('int', None)</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>1e-09</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>python3</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>CPU</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>thread 21587 (python3)</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>[[1], [1]]</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>['int', 'int']</t>
-        </is>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>[[2], [2]]</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>['', '']</t>
-        </is>
-      </c>
-      <c r="AC6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>5</v>
-      </c>
-      <c r="AJ6" t="n">
         <v>23812</v>
       </c>
     </row>
@@ -27319,10 +27179,10 @@
         <v>7.68e-07</v>
       </c>
       <c r="P46" t="n">
-        <v>0.0029296875</v>
+        <v>0.001466751098632812</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.25</v>
+        <v>0.4993498049414825</v>
       </c>
       <c r="R46" t="inlineStr">
         <is>
@@ -27330,10 +27190,10 @@
         </is>
       </c>
       <c r="S46" t="n">
-        <v>0.0009726418028326389</v>
+        <v>0.0004869541317567053</v>
       </c>
       <c r="T46" t="n">
-        <v>7.280491932446589e-05</v>
+        <v>3.644985869825148e-05</v>
       </c>
       <c r="U46" t="n">
         <v>0.0002431604507081597</v>
@@ -27360,13 +27220,13 @@
         <v>38.951</v>
       </c>
       <c r="AC46" t="n">
-        <v>0.0009558318314951775</v>
+        <v>0.0004785382020962185</v>
       </c>
       <c r="AD46" t="n">
-        <v>0.0008651022344448264</v>
+        <v>0.0004331143348229632</v>
       </c>
       <c r="AE46" t="n">
-        <v>0.001078689412773253</v>
+        <v>0.0005400469781397342</v>
       </c>
       <c r="AF46" t="n">
         <v>0.0002389579578737944</v>
@@ -27398,7 +27258,7 @@
       </c>
       <c r="AN46" t="inlineStr">
         <is>
-          <t>{'num_input_elems': 768, 'num_output_elems': 768, 'dtype_in_out': ('c10::BFloat16', None), 'reduce_type': 'norm'}</t>
+          <t>{'num_input_elems': 768, 'num_output_elems': 1, 'dtype_in_out': ('c10::BFloat16', None), 'reduce_type': 'norm'}</t>
         </is>
       </c>
       <c r="AO46" t="b">

</xml_diff>